<commit_message>
fixed bug with SAT_NAMES
</commit_message>
<xml_diff>
--- a/forecasts/forecast_28112025.xlsx
+++ b/forecasts/forecast_28112025.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +76,21 @@
         <fgColor rgb="0000bfff"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006495ed"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ee82ee"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ba55d3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -95,19 +110,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,6 +557,26 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>flight 10</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>flight 11</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>flight 12</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>flight 13</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>name</t>
         </is>
       </c>
@@ -551,37 +589,42 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:33</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>16:22</t>
+          <t>16:17</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>18:23</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>19:05</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>21:01</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>SARAL</t>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>23:31</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>CFOSAT</t>
         </is>
       </c>
     </row>
@@ -593,52 +636,72 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20:34</t>
+          <t>20:33</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>00:41</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>02:11</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>03:36</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>04:14</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>05:35</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>16:57</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>18:21</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>SENTINEL-3A</t>
+          <t>03:46</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>19:32</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>21:28</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>23:44</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>HAIYANG-2B</t>
         </is>
       </c>
     </row>
@@ -650,47 +713,77 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>17:58</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>00:41</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>06:23</t>
+          <t>03:20</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>05:37</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>17:45</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>18:31</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>19:03</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>21:45</t>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>20:19</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
         <is>
-          <t>SENTINEL-3B</t>
+          <t>23:09</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>23:16</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>JASON-3</t>
         </is>
       </c>
     </row>
@@ -702,62 +795,67 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>21:33</t>
+          <t>PD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>17:41</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>04:24</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>04:54</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>09:28</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>12:38</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>18:33</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>19:46</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>20:10</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>20:13</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>22:06</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr">
-        <is>
-          <t>CRYOSAT 2</t>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>00:55</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>03:33</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>07:57</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>23:31</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>23:56</t>
+        </is>
+      </c>
+      <c r="Q5" s="11" t="inlineStr">
+        <is>
+          <t>SARAL</t>
         </is>
       </c>
     </row>
@@ -769,42 +867,57 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>22:20</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18:24</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>03:56</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>05:03</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>06:04</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>19:22</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>20:24</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>SENTINEL-6</t>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>02:22</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>07:57</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>18:28</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>20:48</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>23:53</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>SENTINEL-3A</t>
         </is>
       </c>
     </row>
@@ -816,41 +929,499 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>20:37</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>02:26</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>22:28</t>
-        </is>
-      </c>
-      <c r="M7" s="9" t="inlineStr">
-        <is>
-          <t>SENTINEL-1A</t>
+          <t>03:42</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>06:24</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>07:13</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>19:06</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="Q7" s="6" t="inlineStr">
+        <is>
+          <t>SENTINEL-3B</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>SWOT</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04/12/2025</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>21:04</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>00:15</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>00:20</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>02:59</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>21:17</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>SENTINEL-6A</t>
         </is>
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>05/12/2025</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>21:28</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>17:56</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>00:38</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>00:56</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>04:31</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>06:23</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>SENTINEL-2A</t>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>CRYOSAT 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06/12/2025</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>21:48</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>00:57</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>01:01</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>03:36</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>04:43</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>06:19</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>20:12</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>SENTINEL-1A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07/12/2025</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>00:57</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>01:11</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>01:22</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>05:19</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>06:37</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>08:24</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>15:39</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>20:04</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>20:34</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="Q11" s="7" t="inlineStr">
+        <is>
+          <t>HAIYANG-2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08/12/2025</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>00:58</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>01:45</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>05:32</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>07:09</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>08:42</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>20:19</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="Q12" s="12" t="inlineStr">
+        <is>
+          <t>SWOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>09/12/2025</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>00:58</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>01:27</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>07:13</t>
         </is>
       </c>
     </row>

</xml_diff>